<commit_message>
Skills and Resources Audit
- Skills and Resources Audit
- Updated booked hours
</commit_message>
<xml_diff>
--- a/Documentation/Week 3/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 3/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 3/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1423A34-F8ED-424C-A688-90CBEB1B1869}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45BA7D6D-7C2C-4E33-854F-43D45B03883C}"/>
   <bookViews>
-    <workbookView xWindow="8895" yWindow="5070" windowWidth="22560" windowHeight="12270" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28020" yWindow="900" windowWidth="21600" windowHeight="11235" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="18">
   <si>
     <t>Wk</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>Meeting documentation</t>
+  </si>
+  <si>
+    <t>Skills and Resources Audit</t>
   </si>
 </sst>
 </file>
@@ -330,6 +333,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -348,14 +359,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -793,36 +796,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="16"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -842,7 +845,7 @@
       </c>
       <c r="F3" s="18"/>
       <c r="G3" s="9"/>
-      <c r="H3" s="14"/>
+      <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -872,7 +875,7 @@
         <v>1.2500000000582077</v>
       </c>
       <c r="I4" s="1">
-        <f>((D4+E4)-(B4+C4))*24</f>
+        <f t="shared" ref="I4:I35" si="0">((D4+E4)-(B4+C4))*24</f>
         <v>1.2500000000582077</v>
       </c>
     </row>
@@ -896,7 +899,7 @@
         <v>9</v>
       </c>
       <c r="G5" s="6">
-        <f t="shared" ref="G5:G30" si="0">IF(I5&gt;0,I5,IF(I5=0, " ", "ERROR"))</f>
+        <f t="shared" ref="G5:G30" si="1">IF(I5&gt;0,I5,IF(I5=0, " ", "ERROR"))</f>
         <v>0.99999999994179234</v>
       </c>
       <c r="H5" s="1">
@@ -904,7 +907,7 @@
         <v>2.25</v>
       </c>
       <c r="I5" s="1">
-        <f>((D5+E5)-(B5+C5))*24</f>
+        <f t="shared" si="0"/>
         <v>0.99999999994179234</v>
       </c>
     </row>
@@ -928,15 +931,15 @@
         <v>11</v>
       </c>
       <c r="G6" s="6">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="H6" s="1">
+        <f t="shared" ref="H6:H30" si="2">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
+        <v>3</v>
+      </c>
+      <c r="I6" s="1">
         <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="H6" s="1">
-        <f t="shared" ref="H6:H30" si="1">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
-        <v>3</v>
-      </c>
-      <c r="I6" s="1">
-        <f>((D6+E6)-(B6+C6))*24</f>
         <v>0.75</v>
       </c>
     </row>
@@ -960,15 +963,15 @@
         <v>12</v>
       </c>
       <c r="G7" s="6">
+        <f t="shared" si="1"/>
+        <v>0.99999999994179234</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="2"/>
+        <v>3.9999999999417923</v>
+      </c>
+      <c r="I7" s="1">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
-      </c>
-      <c r="H7" s="1">
-        <f t="shared" si="1"/>
-        <v>3.9999999999417923</v>
-      </c>
-      <c r="I7" s="1">
-        <f>((D7+E7)-(B7+C7))*24</f>
         <v>0.99999999994179234</v>
       </c>
     </row>
@@ -992,15 +995,15 @@
         <v>13</v>
       </c>
       <c r="G8" s="6">
+        <f t="shared" si="1"/>
+        <v>0.50000000005820766</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="2"/>
+        <v>4.5</v>
+      </c>
+      <c r="I8" s="1">
         <f t="shared" si="0"/>
-        <v>0.50000000005820766</v>
-      </c>
-      <c r="H8" s="1">
-        <f t="shared" si="1"/>
-        <v>4.5</v>
-      </c>
-      <c r="I8" s="1">
-        <f>((D8+E8)-(B8+C8))*24</f>
         <v>0.50000000005820766</v>
       </c>
     </row>
@@ -1024,15 +1027,15 @@
         <v>14</v>
       </c>
       <c r="G9" s="6">
+        <f t="shared" si="1"/>
+        <v>0.50000000005820766</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="2"/>
+        <v>5.0000000000582077</v>
+      </c>
+      <c r="I9" s="1">
         <f t="shared" si="0"/>
-        <v>0.50000000005820766</v>
-      </c>
-      <c r="H9" s="1">
-        <f t="shared" si="1"/>
-        <v>5.0000000000582077</v>
-      </c>
-      <c r="I9" s="1">
-        <f>((D9+E9)-(B9+C9))*24</f>
         <v>0.50000000005820766</v>
       </c>
     </row>
@@ -1056,15 +1059,15 @@
         <v>15</v>
       </c>
       <c r="G10" s="6">
+        <f t="shared" si="1"/>
+        <v>1.2500000000582077</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="2"/>
+        <v>6.2500000001164153</v>
+      </c>
+      <c r="I10" s="1">
         <f t="shared" si="0"/>
-        <v>1.2500000000582077</v>
-      </c>
-      <c r="H10" s="1">
-        <f t="shared" si="1"/>
-        <v>6.2500000001164153</v>
-      </c>
-      <c r="I10" s="1">
-        <f>((D10+E10)-(B10+C10))*24</f>
         <v>1.2500000000582077</v>
       </c>
     </row>
@@ -1088,15 +1091,15 @@
         <v>9</v>
       </c>
       <c r="G11" s="6">
+        <f t="shared" si="1"/>
+        <v>0.99999999994179234</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="2"/>
+        <v>7.2500000000582077</v>
+      </c>
+      <c r="I11" s="1">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
-      </c>
-      <c r="H11" s="1">
-        <f t="shared" si="1"/>
-        <v>7.2500000000582077</v>
-      </c>
-      <c r="I11" s="1">
-        <f>((D11+E11)-(B11+C11))*24</f>
         <v>0.99999999994179234</v>
       </c>
     </row>
@@ -1120,15 +1123,15 @@
         <v>12</v>
       </c>
       <c r="G12" s="6">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
+      <c r="H12" s="1">
+        <f t="shared" si="2"/>
+        <v>8.0000000000582077</v>
+      </c>
+      <c r="I12" s="1">
         <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="H12" s="1">
-        <f t="shared" si="1"/>
-        <v>8.0000000000582077</v>
-      </c>
-      <c r="I12" s="1">
-        <f>((D12+E12)-(B12+C12))*24</f>
         <v>0.75</v>
       </c>
     </row>
@@ -1152,34 +1155,48 @@
         <v>16</v>
       </c>
       <c r="G13" s="6">
+        <f t="shared" si="1"/>
+        <v>1.2499999998835847</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" si="2"/>
+        <v>9.2499999999417923</v>
+      </c>
+      <c r="I13" s="1">
         <f t="shared" si="0"/>
         <v>1.2499999998835847</v>
       </c>
-      <c r="H13" s="1">
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>3</v>
+      </c>
+      <c r="B14" s="4">
+        <v>44778</v>
+      </c>
+      <c r="C14" s="5">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D14" s="4">
+        <v>44778</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="6">
         <f t="shared" si="1"/>
-        <v>9.2499999999417923</v>
-      </c>
-      <c r="I13" s="1">
-        <f>((D13+E13)-(B13+C13))*24</f>
-        <v>1.2499999998835847</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="4"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="G14" s="6" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" si="2"/>
+        <v>9.9999999999417923</v>
+      </c>
+      <c r="I14" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H14" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I14" s="1">
-        <f>((D14+E14)-(B14+C14))*24</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1187,16 +1204,19 @@
       <c r="C15" s="5"/>
       <c r="D15" s="4"/>
       <c r="E15" s="5"/>
+      <c r="F15" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="G15" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H15" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I15" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H15" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I15" s="1">
-        <f>((D15+E15)-(B15+C15))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1206,15 +1226,15 @@
       <c r="D16" s="4"/>
       <c r="E16" s="5"/>
       <c r="G16" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H16" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I16" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H16" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I16" s="1">
-        <f>((D16+E16)-(B16+C16))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1224,15 +1244,15 @@
       <c r="D17" s="4"/>
       <c r="E17" s="5"/>
       <c r="G17" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H17" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I17" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H17" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I17" s="1">
-        <f>((D17+E17)-(B17+C17))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1242,15 +1262,15 @@
       <c r="D18" s="4"/>
       <c r="E18" s="5"/>
       <c r="G18" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H18" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I18" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H18" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I18" s="1">
-        <f>((D18+E18)-(B18+C18))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1260,15 +1280,15 @@
       <c r="D19" s="4"/>
       <c r="E19" s="5"/>
       <c r="G19" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H19" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I19" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H19" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I19" s="1">
-        <f>((D19+E19)-(B19+C19))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1278,15 +1298,15 @@
       <c r="D20" s="4"/>
       <c r="E20" s="5"/>
       <c r="G20" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H20" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I20" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H20" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I20" s="1">
-        <f>((D20+E20)-(B20+C20))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1296,15 +1316,15 @@
       <c r="D21" s="4"/>
       <c r="E21" s="5"/>
       <c r="G21" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H21" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I21" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H21" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I21" s="1">
-        <f>((D21+E21)-(B21+C21))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1314,15 +1334,15 @@
       <c r="D22" s="4"/>
       <c r="E22" s="5"/>
       <c r="G22" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H22" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I22" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H22" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I22" s="1">
-        <f>((D22+E22)-(B22+C22))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1332,15 +1352,15 @@
       <c r="D23" s="4"/>
       <c r="E23" s="5"/>
       <c r="G23" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H23" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I23" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H23" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I23" s="1">
-        <f>((D23+E23)-(B23+C23))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1350,15 +1370,15 @@
       <c r="D24" s="4"/>
       <c r="E24" s="5"/>
       <c r="G24" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H24" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I24" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H24" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I24" s="1">
-        <f>((D24+E24)-(B24+C24))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1368,15 +1388,15 @@
       <c r="D25" s="4"/>
       <c r="E25" s="5"/>
       <c r="G25" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H25" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I25" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H25" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I25" s="1">
-        <f>((D25+E25)-(B25+C25))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1386,15 +1406,15 @@
       <c r="D26" s="4"/>
       <c r="E26" s="5"/>
       <c r="G26" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H26" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I26" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H26" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I26" s="1">
-        <f>((D26+E26)-(B26+C26))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1404,15 +1424,15 @@
       <c r="D27" s="4"/>
       <c r="E27" s="5"/>
       <c r="G27" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H27" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I27" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H27" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I27" s="1">
-        <f>((D27+E27)-(B27+C27))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1422,15 +1442,15 @@
       <c r="D28" s="4"/>
       <c r="E28" s="5"/>
       <c r="G28" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H28" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I28" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H28" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I28" s="1">
-        <f>((D28+E28)-(B28+C28))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1440,15 +1460,15 @@
       <c r="D29" s="4"/>
       <c r="E29" s="5"/>
       <c r="G29" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H29" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I29" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H29" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I29" s="1">
-        <f>((D29+E29)-(B29+C29))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1458,15 +1478,15 @@
       <c r="D30" s="4"/>
       <c r="E30" s="5"/>
       <c r="G30" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H30" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="I30" s="1">
         <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H30" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="I30" s="1">
-        <f>((D30+E30)-(B30+C30))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1474,14 +1494,14 @@
       <c r="A31" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
@@ -1492,7 +1512,7 @@
         <v>6</v>
       </c>
       <c r="I31" s="1" t="e">
-        <f>((D31+E31)-(B31+C31))*24</f>
+        <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -1514,7 +1534,7 @@
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
       <c r="I32" s="1" t="e">
-        <f>((D32+E32)-(B32+C32))*24</f>
+        <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -1524,7 +1544,7 @@
       <c r="D33" s="4"/>
       <c r="E33" s="5"/>
       <c r="G33" s="6" t="str">
-        <f t="shared" ref="G33:G64" si="2">IF(I33&gt;0,I33,IF(I33=0, " ", "ERROR"))</f>
+        <f t="shared" ref="G33:G64" si="3">IF(I33&gt;0,I33,IF(I33=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H33" s="1" t="str">
@@ -1532,7 +1552,7 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="I33" s="1">
-        <f>((D33+E33)-(B33+C33))*24</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1542,15 +1562,15 @@
       <c r="D34" s="4"/>
       <c r="E34" s="5"/>
       <c r="G34" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H34" s="1" t="str">
-        <f t="shared" ref="H34:H64" si="3">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
+        <f t="shared" ref="H34:H64" si="4">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I34" s="1">
-        <f>((D34+E34)-(B34+C34))*24</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1560,15 +1580,15 @@
       <c r="D35" s="4"/>
       <c r="E35" s="5"/>
       <c r="G35" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H35" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I35" s="1">
-        <f>((D35+E35)-(B35+C35))*24</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1578,15 +1598,15 @@
       <c r="D36" s="4"/>
       <c r="E36" s="5"/>
       <c r="G36" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H36" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I36" s="1">
-        <f>((D36+E36)-(B36+C36))*24</f>
+        <f t="shared" ref="I36:I68" si="5">((D36+E36)-(B36+C36))*24</f>
         <v>0</v>
       </c>
     </row>
@@ -1596,15 +1616,15 @@
       <c r="D37" s="4"/>
       <c r="E37" s="5"/>
       <c r="G37" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H37" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I37" s="1">
-        <f>((D37+E37)-(B37+C37))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1614,15 +1634,15 @@
       <c r="D38" s="4"/>
       <c r="E38" s="5"/>
       <c r="G38" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H38" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I38" s="1">
-        <f>((D38+E38)-(B38+C38))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1632,15 +1652,15 @@
       <c r="D39" s="4"/>
       <c r="E39" s="5"/>
       <c r="G39" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H39" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I39" s="1">
-        <f>((D39+E39)-(B39+C39))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1650,15 +1670,15 @@
       <c r="D40" s="4"/>
       <c r="E40" s="5"/>
       <c r="G40" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H40" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I40" s="1">
-        <f>((D40+E40)-(B40+C40))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1668,15 +1688,15 @@
       <c r="D41" s="4"/>
       <c r="E41" s="5"/>
       <c r="G41" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H41" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I41" s="1">
-        <f>((D41+E41)-(B41+C41))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1686,15 +1706,15 @@
       <c r="D42" s="4"/>
       <c r="E42" s="5"/>
       <c r="G42" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H42" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I42" s="1">
-        <f>((D42+E42)-(B42+C42))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1704,15 +1724,15 @@
       <c r="D43" s="4"/>
       <c r="E43" s="5"/>
       <c r="G43" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H43" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I43" s="1">
-        <f>((D43+E43)-(B43+C43))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1722,15 +1742,15 @@
       <c r="D44" s="4"/>
       <c r="E44" s="5"/>
       <c r="G44" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H44" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I44" s="1">
-        <f>((D44+E44)-(B44+C44))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1740,15 +1760,15 @@
       <c r="D45" s="4"/>
       <c r="E45" s="5"/>
       <c r="G45" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H45" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I45" s="1">
-        <f>((D45+E45)-(B45+C45))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1758,15 +1778,15 @@
       <c r="D46" s="4"/>
       <c r="E46" s="5"/>
       <c r="G46" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H46" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I46" s="1">
-        <f>((D46+E46)-(B46+C46))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1776,15 +1796,15 @@
       <c r="D47" s="4"/>
       <c r="E47" s="5"/>
       <c r="G47" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H47" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I47" s="1">
-        <f>((D47+E47)-(B47+C47))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1794,15 +1814,15 @@
       <c r="D48" s="4"/>
       <c r="E48" s="5"/>
       <c r="G48" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H48" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I48" s="1">
-        <f>((D48+E48)-(B48+C48))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1812,15 +1832,15 @@
       <c r="D49" s="4"/>
       <c r="E49" s="5"/>
       <c r="G49" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H49" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I49" s="1">
-        <f>((D49+E49)-(B49+C49))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1830,15 +1850,15 @@
       <c r="D50" s="4"/>
       <c r="E50" s="5"/>
       <c r="G50" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H50" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I50" s="1">
-        <f>((D50+E50)-(B50+C50))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1848,15 +1868,15 @@
       <c r="D51" s="4"/>
       <c r="E51" s="5"/>
       <c r="G51" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H51" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I51" s="1">
-        <f>((D51+E51)-(B51+C51))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1866,15 +1886,15 @@
       <c r="D52" s="4"/>
       <c r="E52" s="5"/>
       <c r="G52" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H52" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I52" s="1">
-        <f>((D52+E52)-(B52+C52))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1884,15 +1904,15 @@
       <c r="D53" s="4"/>
       <c r="E53" s="5"/>
       <c r="G53" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H53" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I53" s="1">
-        <f>((D53+E53)-(B53+C53))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1902,15 +1922,15 @@
       <c r="D54" s="4"/>
       <c r="E54" s="5"/>
       <c r="G54" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H54" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I54" s="1">
-        <f>((D54+E54)-(B54+C54))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1920,15 +1940,15 @@
       <c r="D55" s="4"/>
       <c r="E55" s="5"/>
       <c r="G55" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H55" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I55" s="1">
-        <f>((D55+E55)-(B55+C55))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1938,15 +1958,15 @@
       <c r="D56" s="4"/>
       <c r="E56" s="5"/>
       <c r="G56" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H56" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I56" s="1">
-        <f>((D56+E56)-(B56+C56))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1956,15 +1976,15 @@
       <c r="D57" s="4"/>
       <c r="E57" s="5"/>
       <c r="G57" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H57" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I57" s="1">
-        <f>((D57+E57)-(B57+C57))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1974,15 +1994,15 @@
       <c r="D58" s="4"/>
       <c r="E58" s="5"/>
       <c r="G58" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H58" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I58" s="1">
-        <f>((D58+E58)-(B58+C58))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -1992,90 +2012,90 @@
       <c r="D59" s="4"/>
       <c r="E59" s="5"/>
       <c r="G59" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H59" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I59" s="1">
-        <f>((D59+E59)-(B59+C59))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="60" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B60" s="4"/>
       <c r="G60" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H60" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I60" s="1">
-        <f>((D60+E60)-(B60+C60))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="4"/>
       <c r="G61" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H61" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I61" s="1">
-        <f>((D61+E61)-(B61+C61))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B62" s="4"/>
       <c r="G62" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H62" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I62" s="1">
-        <f>((D62+E62)-(B62+C62))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B63" s="4"/>
       <c r="G63" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H63" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I63" s="1">
-        <f>((D63+E63)-(B63+C63))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="64" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B64" s="4"/>
       <c r="G64" s="6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H64" s="1" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I64" s="1">
-        <f>((D64+E64)-(B64+C64))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -2083,14 +2103,14 @@
       <c r="A65" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="B65" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="15" t="s">
+      <c r="C65" s="11"/>
+      <c r="D65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="16"/>
+      <c r="E65" s="11"/>
       <c r="F65" s="7" t="s">
         <v>5</v>
       </c>
@@ -2101,7 +2121,7 @@
         <v>6</v>
       </c>
       <c r="I65" s="1" t="e">
-        <f>((D65+E65)-(B65+C65))*24</f>
+        <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -2123,13 +2143,13 @@
       <c r="G66" s="7"/>
       <c r="H66" s="7"/>
       <c r="I66" s="1" t="e">
-        <f>((D66+E66)-(B66+C66))*24</f>
+        <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G67" s="6" t="str">
-        <f t="shared" ref="G67:G98" si="4">IF(I67&gt;0,I67,IF(I67=0, " ", "ERROR"))</f>
+        <f t="shared" ref="G67:G98" si="6">IF(I67&gt;0,I67,IF(I67=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H67" s="1" t="str">
@@ -2137,441 +2157,441 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="I67" s="1">
-        <f>((D67+E67)-(B67+C67))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G68" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H68" s="1" t="str">
-        <f t="shared" ref="H68:H98" si="5">IF(AND(G68&lt;&gt;" ",G68&lt;&gt;"ERROR",H67&lt;&gt;" ", H67&lt;&gt;"ERROR"),G68+H67," ")</f>
+        <f t="shared" ref="H68:H98" si="7">IF(AND(G68&lt;&gt;" ",G68&lt;&gt;"ERROR",H67&lt;&gt;" ", H67&lt;&gt;"ERROR"),G68+H67," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I68" s="1">
-        <f>((D68+E68)-(B68+C68))*24</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G69" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H69" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I69" s="1">
-        <f t="shared" ref="I69:I132" si="6">((D69+E69)-(B69+C69))*24</f>
+        <f t="shared" ref="I69:I132" si="8">((D69+E69)-(B69+C69))*24</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G70" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H70" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I70" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G71" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H71" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I71" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G72" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H72" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I72" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G73" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H73" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I73" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G74" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H74" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I74" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G75" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H75" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I75" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G76" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H76" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I76" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G77" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H77" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I77" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G78" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H78" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I78" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G79" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H79" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I79" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G80" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H80" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I80" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="81" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G81" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H81" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I81" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="82" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G82" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H82" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I82" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="83" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G83" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H83" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I83" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="84" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G84" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H84" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I84" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="85" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G85" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H85" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I85" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="86" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G86" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H86" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I86" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="87" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G87" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H87" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I87" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="88" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G88" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H88" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I88" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="89" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G89" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H89" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I89" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="90" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G90" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H90" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I90" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="91" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G91" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H91" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I91" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="92" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G92" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H92" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I92" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="93" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G93" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H93" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I93" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="94" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G94" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H94" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I94" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="95" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G95" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H95" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I95" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="96" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G96" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H96" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I96" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G97" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H97" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I97" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G98" s="6" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H98" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I98" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2579,14 +2599,14 @@
       <c r="A99" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="15" t="s">
+      <c r="B99" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15" t="s">
+      <c r="C99" s="11"/>
+      <c r="D99" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E99" s="16"/>
+      <c r="E99" s="11"/>
       <c r="F99" s="7" t="s">
         <v>5</v>
       </c>
@@ -2597,7 +2617,7 @@
         <v>6</v>
       </c>
       <c r="I99" s="1" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -2619,13 +2639,13 @@
       <c r="G100" s="7"/>
       <c r="H100" s="7"/>
       <c r="I100" s="1" t="e">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G101" s="6" t="str">
-        <f t="shared" ref="G101:G132" si="7">IF(I101&gt;0,I101,IF(I101=0, " ", "ERROR"))</f>
+        <f t="shared" ref="G101:G132" si="9">IF(I101&gt;0,I101,IF(I101=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H101" s="1" t="str">
@@ -2633,458 +2653,446 @@
         <v xml:space="preserve"> </v>
       </c>
       <c r="I101" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G102" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H102" s="1" t="str">
-        <f t="shared" ref="H102:H132" si="8">IF(AND(G102&lt;&gt;" ",G102&lt;&gt;"ERROR",H101&lt;&gt;" ", H101&lt;&gt;"ERROR"),G102+H101," ")</f>
+        <f t="shared" ref="H102:H132" si="10">IF(AND(G102&lt;&gt;" ",G102&lt;&gt;"ERROR",H101&lt;&gt;" ", H101&lt;&gt;"ERROR"),G102+H101," ")</f>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I102" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G103" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H103" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I103" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G104" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H104" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I104" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G105" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H105" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I105" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G106" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H106" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I106" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G107" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H107" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I107" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G108" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H108" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I108" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G109" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H109" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I109" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G110" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H110" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I110" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G111" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H111" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I111" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G112" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H112" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I112" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="113" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G113" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H113" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I113" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="114" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G114" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H114" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I114" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="115" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G115" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H115" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I115" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="116" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G116" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H116" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I116" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="117" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G117" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H117" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I117" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="118" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G118" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H118" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I118" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="119" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G119" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H119" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I119" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="120" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G120" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H120" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I120" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="121" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G121" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H121" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I121" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="122" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G122" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H122" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I122" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="123" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G123" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H123" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I123" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="124" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G124" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H124" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I124" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="125" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G125" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H125" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I125" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="126" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G126" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H126" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I126" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="127" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G127" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H127" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I127" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="128" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G128" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H128" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I128" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="129" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G129" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H129" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I129" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="130" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G130" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H130" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I130" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="131" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G131" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H131" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I131" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
     <row r="132" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G132" s="6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="H132" s="1" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v xml:space="preserve"> </v>
       </c>
       <c r="I132" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -3098,6 +3106,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>

<commit_message>
Meeting Agenda Updated and Timesheet explained
</commit_message>
<xml_diff>
--- a/Documentation/Week 3/Booked Hours/Booked_Hours_Christo.xlsx
+++ b/Documentation/Week 3/Booked Hours/Booked_Hours_Christo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24432207_student_uwa_edu_au/Documents/UWA - Student/2026_Sem2/CITS3200 - Professional Computing/Project/Repo/CITS3200_Project/Documentation/Week 3/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D59B9C88-7AB3-4C47-B355-0FCD75E99A07}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:40009_{31A31D98-CA30-574B-8C94-F50C456CB544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3155B74-B22C-4FFA-B6C8-21BC7D6D98A2}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1500" windowWidth="17280" windowHeight="12132" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
@@ -333,6 +333,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
@@ -351,14 +359,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -792,36 +792,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="12"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="14"/>
     </row>
     <row r="2" spans="1:9" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="15" t="s">
+      <c r="C2" s="11"/>
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="16"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>6</v>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="F3" s="18"/>
       <c r="G3" s="9"/>
-      <c r="H3" s="14"/>
+      <c r="H3" s="16"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
@@ -1501,14 +1501,14 @@
       <c r="A31" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B31" s="15" t="s">
+      <c r="B31" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="15" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E31" s="16"/>
+      <c r="E31" s="11"/>
       <c r="F31" s="7" t="s">
         <v>5</v>
       </c>
@@ -2110,14 +2110,14 @@
       <c r="A65" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B65" s="15" t="s">
+      <c r="B65" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C65" s="16"/>
-      <c r="D65" s="15" t="s">
+      <c r="C65" s="11"/>
+      <c r="D65" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E65" s="16"/>
+      <c r="E65" s="11"/>
       <c r="F65" s="7" t="s">
         <v>5</v>
       </c>
@@ -2606,14 +2606,14 @@
       <c r="A99" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="15" t="s">
+      <c r="B99" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="16"/>
-      <c r="D99" s="15" t="s">
+      <c r="C99" s="11"/>
+      <c r="D99" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E99" s="16"/>
+      <c r="E99" s="11"/>
       <c r="F99" s="7" t="s">
         <v>5</v>
       </c>
@@ -3100,18 +3100,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="D99:E99"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G99:G100"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:E65"/>
-    <mergeCell ref="F65:F66"/>
     <mergeCell ref="H31:H32"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="A1:H1"/>
@@ -3125,6 +3113,18 @@
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:E65"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="H99:H100"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="D99:E99"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G99:G100"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>